<commit_message>
added new VOs and run checklist and apply changes
</commit_message>
<xml_diff>
--- a/MTG2A04_L01_S01_VO_MANIFEST.xlsx
+++ b/MTG2A04_L01_S01_VO_MANIFEST.xlsx
@@ -629,11 +629,11 @@
       </c>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n">
-        <v>9.73</v>
+        <v>9.66</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Transition «चलिए, शुरू करते हैं।»</t>
+          <t>Transition «चलिए, शुरू करें!»</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
@@ -661,7 +661,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए और मेरे साथ जानिए। चलिए, शुरू करते हैं।</t>
+          <t>ध्यान से देखिए और मेरे साथ जानिए। चलिए, शुरू करें!</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -676,11 +676,11 @@
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n">
-        <v>4.13</v>
+        <v>4.24</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -723,11 +723,11 @@
       </c>
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="n">
-        <v>2.01</v>
+        <v>1.73</v>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record - DRAFT script, SME to finalise</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -770,11 +770,11 @@
       </c>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n">
-        <v>2.01</v>
+        <v>2.43</v>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record - DRAFT script, SME to finalise</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -817,11 +817,11 @@
       </c>
       <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n">
-        <v>5.65</v>
+        <v>5.12</v>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -864,11 +864,11 @@
       </c>
       <c r="I10" s="8" t="n"/>
       <c r="J10" s="8" t="n">
-        <v>2.33</v>
+        <v>2.02</v>
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -915,11 +915,11 @@
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>1.09</v>
+        <v>1.17</v>
       </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -962,11 +962,11 @@
       </c>
       <c r="I12" s="6" t="n"/>
       <c r="J12" s="6" t="n">
-        <v>2.37</v>
+        <v>2.46</v>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1013,11 +1013,11 @@
         </is>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1.09</v>
+        <v>1.17</v>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1060,11 +1060,11 @@
       </c>
       <c r="I14" s="8" t="n"/>
       <c r="J14" s="8" t="n">
-        <v>4.69</v>
+        <v>4.67</v>
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1107,11 +1107,11 @@
       </c>
       <c r="I15" s="8" t="n"/>
       <c r="J15" s="8" t="n">
-        <v>4.29</v>
+        <v>3.64</v>
       </c>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1154,11 +1154,11 @@
       </c>
       <c r="I16" s="8" t="n"/>
       <c r="J16" s="8" t="n">
-        <v>7.17</v>
+        <v>6.61</v>
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1201,11 +1201,11 @@
       </c>
       <c r="I17" s="6" t="n"/>
       <c r="J17" s="6" t="n">
-        <v>3.77</v>
+        <v>3.62</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1252,11 +1252,11 @@
         </is>
       </c>
       <c r="J18" s="6" t="n">
-        <v>4.89</v>
+        <v>4.54</v>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1303,11 +1303,11 @@
         </is>
       </c>
       <c r="J19" s="6" t="n">
-        <v>3.17</v>
+        <v>4.26</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1350,11 +1350,11 @@
       </c>
       <c r="I20" s="6" t="n"/>
       <c r="J20" s="6" t="n">
-        <v>6.81</v>
+        <v>6.48</v>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1397,11 +1397,11 @@
       </c>
       <c r="I21" s="8" t="n"/>
       <c r="J21" s="8" t="n">
-        <v>4.05</v>
+        <v>3.64</v>
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record - EAR-CHECK</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1444,11 +1444,11 @@
       </c>
       <c r="I22" s="8" t="n"/>
       <c r="J22" s="8" t="n">
-        <v>4.09</v>
+        <v>4.35</v>
       </c>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1491,11 +1491,11 @@
       </c>
       <c r="I23" s="8" t="n"/>
       <c r="J23" s="8" t="n">
-        <v>4.69</v>
+        <v>4.47</v>
       </c>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1538,11 +1538,11 @@
       </c>
       <c r="I24" s="8" t="n"/>
       <c r="J24" s="8" t="n">
-        <v>4.21</v>
+        <v>4.89</v>
       </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1589,11 +1589,11 @@
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>4.89</v>
+        <v>4.54</v>
       </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1640,11 +1640,11 @@
         </is>
       </c>
       <c r="J26" s="8" t="n">
-        <v>3.17</v>
+        <v>4.26</v>
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1687,11 +1687,11 @@
       </c>
       <c r="I27" s="8" t="n"/>
       <c r="J27" s="8" t="n">
-        <v>7.01</v>
+        <v>6.96</v>
       </c>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1734,11 +1734,11 @@
       </c>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n">
-        <v>2.53</v>
+        <v>1.78</v>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1781,11 +1781,11 @@
       </c>
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="6" t="n">
-        <v>3.89</v>
+        <v>4.31</v>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1875,11 +1875,11 @@
       </c>
       <c r="I31" s="6" t="n"/>
       <c r="J31" s="6" t="n">
-        <v>1.45</v>
+        <v>1.18</v>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1922,11 +1922,11 @@
       </c>
       <c r="I32" s="6" t="n"/>
       <c r="J32" s="6" t="n">
-        <v>3.53</v>
+        <v>3.82</v>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -1969,11 +1969,11 @@
       </c>
       <c r="I33" s="6" t="n"/>
       <c r="J33" s="6" t="n">
-        <v>4.21</v>
+        <v>4.26</v>
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2016,11 +2016,11 @@
       </c>
       <c r="I34" s="6" t="n"/>
       <c r="J34" s="6" t="n">
-        <v>3.81</v>
+        <v>3.92</v>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2063,11 +2063,11 @@
       </c>
       <c r="I35" s="6" t="n"/>
       <c r="J35" s="6" t="n">
-        <v>4.69</v>
+        <v>4.05</v>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2110,11 +2110,11 @@
       </c>
       <c r="I36" s="6" t="n"/>
       <c r="J36" s="6" t="n">
-        <v>3.69</v>
+        <v>3.34</v>
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2157,11 +2157,11 @@
       </c>
       <c r="I37" s="6" t="n"/>
       <c r="J37" s="6" t="n">
-        <v>4.45</v>
+        <v>4.49</v>
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2204,11 +2204,11 @@
       </c>
       <c r="I38" s="6" t="n"/>
       <c r="J38" s="6" t="n">
-        <v>3.65</v>
+        <v>3.45</v>
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2251,11 +2251,11 @@
       </c>
       <c r="I39" s="6" t="n"/>
       <c r="J39" s="6" t="n">
-        <v>3.17</v>
+        <v>3.14</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2298,11 +2298,11 @@
       </c>
       <c r="I40" s="6" t="n"/>
       <c r="J40" s="6" t="n">
-        <v>2.97</v>
+        <v>3.61</v>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2345,11 +2345,11 @@
       </c>
       <c r="I41" s="6" t="n"/>
       <c r="J41" s="6" t="n">
-        <v>3.21</v>
+        <v>3.52</v>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2392,11 +2392,11 @@
       </c>
       <c r="I42" s="6" t="n"/>
       <c r="J42" s="6" t="n">
-        <v>3.85</v>
+        <v>4.01</v>
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2439,11 +2439,11 @@
       </c>
       <c r="I43" s="6" t="n"/>
       <c r="J43" s="6" t="n">
-        <v>1.25</v>
+        <v>1.31</v>
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2537,11 +2537,11 @@
         </is>
       </c>
       <c r="J45" s="6" t="n">
-        <v>1.09</v>
+        <v>1.17</v>
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2584,11 +2584,11 @@
       </c>
       <c r="I46" s="6" t="n"/>
       <c r="J46" s="6" t="n">
-        <v>3.93</v>
+        <v>3.3</v>
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2631,11 +2631,11 @@
       </c>
       <c r="I47" s="8" t="n"/>
       <c r="J47" s="8" t="n">
-        <v>2.94</v>
+        <v>2.96</v>
       </c>
       <c r="K47" s="8" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2738,11 +2738,11 @@
         </is>
       </c>
       <c r="F5" s="10" t="n">
-        <v>9.73</v>
+        <v>9.66</v>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए और मेरे साथ जानिए। चलिए, शुरू करते हैं।</t>
+          <t>ध्यान से देखिए और मेरे साथ जानिए। चलिए, शुरू करें!</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -2771,11 +2771,11 @@
         </is>
       </c>
       <c r="F6" s="10" t="n">
-        <v>4.13</v>
+        <v>4.24</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2804,11 +2804,11 @@
         </is>
       </c>
       <c r="F7" s="10" t="n">
-        <v>2.01</v>
+        <v>1.73</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record - DRAFT script, SME to finalise</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2837,11 +2837,11 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>2.01</v>
+        <v>2.43</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record - DRAFT script, SME to finalise</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2870,11 +2870,11 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>5.65</v>
+        <v>5.12</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2903,11 +2903,11 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>2.33</v>
+        <v>2.02</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2936,11 +2936,11 @@
         </is>
       </c>
       <c r="F11" s="10" t="n">
-        <v>1.09</v>
+        <v>1.17</v>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -2969,11 +2969,11 @@
         </is>
       </c>
       <c r="F12" s="10" t="n">
-        <v>2.37</v>
+        <v>2.46</v>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3002,11 +3002,11 @@
         </is>
       </c>
       <c r="F13" s="10" t="n">
-        <v>4.69</v>
+        <v>4.67</v>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3035,11 +3035,11 @@
         </is>
       </c>
       <c r="F14" s="10" t="n">
-        <v>4.29</v>
+        <v>3.64</v>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3068,11 +3068,11 @@
         </is>
       </c>
       <c r="F15" s="10" t="n">
-        <v>7.17</v>
+        <v>6.61</v>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3101,11 +3101,11 @@
         </is>
       </c>
       <c r="F16" s="10" t="n">
-        <v>3.77</v>
+        <v>3.62</v>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3134,11 +3134,11 @@
         </is>
       </c>
       <c r="F17" s="10" t="n">
-        <v>4.89</v>
+        <v>4.54</v>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3167,11 +3167,11 @@
         </is>
       </c>
       <c r="F18" s="10" t="n">
-        <v>3.17</v>
+        <v>4.26</v>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3200,11 +3200,11 @@
         </is>
       </c>
       <c r="F19" s="10" t="n">
-        <v>6.81</v>
+        <v>6.48</v>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3233,11 +3233,11 @@
         </is>
       </c>
       <c r="F20" s="10" t="n">
-        <v>4.05</v>
+        <v>3.64</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record - EAR-CHECK</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3266,11 +3266,11 @@
         </is>
       </c>
       <c r="F21" s="10" t="n">
-        <v>4.09</v>
+        <v>4.35</v>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3299,11 +3299,11 @@
         </is>
       </c>
       <c r="F22" s="10" t="n">
-        <v>4.69</v>
+        <v>4.47</v>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3332,11 +3332,11 @@
         </is>
       </c>
       <c r="F23" s="10" t="n">
-        <v>4.21</v>
+        <v>4.89</v>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3365,11 +3365,11 @@
         </is>
       </c>
       <c r="F24" s="10" t="n">
-        <v>7.01</v>
+        <v>6.96</v>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3398,11 +3398,11 @@
         </is>
       </c>
       <c r="F25" s="10" t="n">
-        <v>2.53</v>
+        <v>1.78</v>
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3431,11 +3431,11 @@
         </is>
       </c>
       <c r="F26" s="10" t="n">
-        <v>3.89</v>
+        <v>4.31</v>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3497,11 +3497,11 @@
         </is>
       </c>
       <c r="F28" s="10" t="n">
-        <v>1.45</v>
+        <v>1.18</v>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3530,11 +3530,11 @@
         </is>
       </c>
       <c r="F29" s="10" t="n">
-        <v>3.53</v>
+        <v>3.82</v>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3563,11 +3563,11 @@
         </is>
       </c>
       <c r="F30" s="10" t="n">
-        <v>4.21</v>
+        <v>4.26</v>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3596,11 +3596,11 @@
         </is>
       </c>
       <c r="F31" s="10" t="n">
-        <v>3.81</v>
+        <v>3.92</v>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3629,11 +3629,11 @@
         </is>
       </c>
       <c r="F32" s="10" t="n">
-        <v>4.69</v>
+        <v>4.05</v>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3662,11 +3662,11 @@
         </is>
       </c>
       <c r="F33" s="10" t="n">
-        <v>3.69</v>
+        <v>3.34</v>
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3695,11 +3695,11 @@
         </is>
       </c>
       <c r="F34" s="10" t="n">
-        <v>4.45</v>
+        <v>4.49</v>
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3728,11 +3728,11 @@
         </is>
       </c>
       <c r="F35" s="10" t="n">
-        <v>3.65</v>
+        <v>3.45</v>
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3761,11 +3761,11 @@
         </is>
       </c>
       <c r="F36" s="10" t="n">
-        <v>3.17</v>
+        <v>3.14</v>
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3794,11 +3794,11 @@
         </is>
       </c>
       <c r="F37" s="10" t="n">
-        <v>2.97</v>
+        <v>3.61</v>
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3827,11 +3827,11 @@
         </is>
       </c>
       <c r="F38" s="10" t="n">
-        <v>3.21</v>
+        <v>3.52</v>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3860,11 +3860,11 @@
         </is>
       </c>
       <c r="F39" s="10" t="n">
-        <v>3.85</v>
+        <v>4.01</v>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3893,11 +3893,11 @@
         </is>
       </c>
       <c r="F40" s="10" t="n">
-        <v>1.25</v>
+        <v>1.31</v>
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3959,11 +3959,11 @@
         </is>
       </c>
       <c r="F42" s="10" t="n">
-        <v>3.93</v>
+        <v>3.3</v>
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -3992,11 +3992,11 @@
         </is>
       </c>
       <c r="F43" s="10" t="n">
-        <v>2.94</v>
+        <v>2.96</v>
       </c>
       <c r="G43" s="10" t="inlineStr">
         <is>
-          <t>TTS placeholder - to record</t>
+          <t>Recorded (SME, 2026-10-21)</t>
         </is>
       </c>
     </row>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>All 39 are Gemini text-to-speech placeholders (voice Leda), so the game is playable now - every one is to be replaced by the final recording.</t>
+          <t>39 of 39 are the SME's recordings (assets/Audio/voiceovers/&lt;id&gt;.wav, trimmed and levelled into assets/Audio/&lt;id&gt;.ogg by scripts/prepare_vo.py); the rest are Gemini TTS placeholders (voice Leda).</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>PYTHONUTF8=1 python scripts/gen_vo_manifest.py   (generated 2026-10-19)</t>
+          <t>PYTHONUTF8=1 python scripts/gen_vo_manifest.py   (generated 2026-10-21)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added new title page VO
</commit_message>
<xml_diff>
--- a/MTG2A04_L01_S01_VO_MANIFEST.xlsx
+++ b/MTG2A04_L01_S01_VO_MANIFEST.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>नमस्ते दोस्त! मैं हूँ स्विफ्टी। परी के स्कूल में पिकनिक होने वाली है। उसे पिकनिक के लिए कुछ सामान खरीदना है। चलिए, उसकी मदद करते हैं!</t>
+          <t>नमस्ते दोस्त! मैं हूँ स्विफ्टी। आज परी बाज़ार जा रही है। उसे कुछ सामान खरीदना है। आइए, हम भी उसके साथ चलते हैं और उसकी मदद करते हैं।</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -629,11 +629,11 @@
       </c>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n">
-        <v>9.66</v>
+        <v>10.31</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Recorded (SME, 2026-10-21)</t>
+          <t>Recorded (SME, 2026-10-22)</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>नमस्ते दोस्त! मैं हूँ स्विफ्टी। परी के स्कूल में पिकनिक होने वाली है। उसे पिकनिक के लिए कुछ सामान खरीदना है। चलिए, उसकी मदद करते हैं!</t>
+          <t>नमस्ते दोस्त! मैं हूँ स्विफ्टी। आज परी बाज़ार जा रही है। उसे कुछ सामान खरीदना है। आइए, हम भी उसके साथ चलते हैं और उसकी मदद करते हैं।</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -2738,11 +2738,11 @@
         </is>
       </c>
       <c r="F5" s="10" t="n">
-        <v>9.66</v>
+        <v>10.31</v>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Recorded (SME, 2026-10-21)</t>
+          <t>Recorded (SME, 2026-10-22)</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>PYTHONUTF8=1 python scripts/gen_vo_manifest.py   (generated 2026-10-21)</t>
+          <t>PYTHONUTF8=1 python scripts/gen_vo_manifest.py   (generated 2026-10-22)</t>
         </is>
       </c>
     </row>

</xml_diff>